<commit_message>
4. **Explore Semantic Relationships**
</commit_message>
<xml_diff>
--- a/projects/project-3/assignment/src/data/bfo-class-axioms.xlsx
+++ b/projects/project-3/assignment/src/data/bfo-class-axioms.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C262"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,7 +446,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b91</t>
+          <t>continuant</t>
         </is>
       </c>
     </row>
@@ -480,1163 +480,4393 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000001</t>
+          <t>n02f2337a1565431a8be6a3d794e45186b91</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000140</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000002</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>continuant fiat boundary</t>
+          <t>continuant</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b145</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000001</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000140</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000002</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>continuant fiat boundary</t>
+          <t>continuant</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000141</t>
+          <t>008-BFO</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000140</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000002</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>continuant fiat boundary</t>
+          <t>continuant</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b146</t>
+          <t>(Elucidation) A continuant is an entity that persists, endures, or continues to exist through time while maintaining its identity</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000016</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000002</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>disposition</t>
+          <t>continuant</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000023</t>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000016</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000002</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>disposition</t>
+          <t>continuant</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000017</t>
+          <t>A human being; a tennis ball; a cave; a region of space; someone's temperature</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000142</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000140</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>fiat line</t>
+          <t>continuant fiat boundary</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000140</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000141</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000142</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000140</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>fiat line</t>
+          <t>continuant fiat boundary</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b147</t>
+          <t>(Elucidation) A continuant fiat boundary b is an immaterial entity that is of zero, one or two dimensions &amp; such that there is no time t when b has a spatial region as continuant part &amp; whose location is determined in relation to some material entity</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000024</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000140</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>fiat object part</t>
+          <t>continuant fiat boundary</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000040</t>
+          <t>continuant fiat boundary</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000147</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000140</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>fiat point</t>
+          <t>continuant fiat boundary</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000140</t>
+          <t>As for fiat point, fiat line, fiat surface</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000147</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000140</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>fiat point</t>
+          <t>continuant fiat boundary</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b152</t>
+          <t>n02f2337a1565431a8be6a3d794e45186b146</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000146</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000140</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>fiat surface</t>
+          <t>continuant fiat boundary</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b151</t>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000146</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000140</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>fiat surface</t>
+          <t>continuant fiat boundary</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000140</t>
+          <t>029-BFO</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000034</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000140</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>function</t>
+          <t>continuant fiat boundary</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000016</t>
+          <t>n02f2337a1565431a8be6a3d794e45186b145</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000031</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000016</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>generically dependent continuant</t>
+          <t>disposition</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000002</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000023</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000182</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000016</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>history</t>
+          <t>disposition</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000015</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000017</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000141</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000016</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>immaterial entity</t>
+          <t>disposition</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000004</t>
+          <t>internally-grounded realizable entity</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000004</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000016</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>independent continuant</t>
+          <t>disposition</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b92</t>
+          <t>disposition</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000004</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000016</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>independent continuant</t>
+          <t>disposition</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000002</t>
+          <t>062-BFO</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000040</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000016</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>material entity</t>
+          <t>disposition</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000004</t>
+          <t>An atom of element X has the disposition to decay to an atom of element Y; the cell wall is disposed to transport cellular material through endocytosis and exocytosis; certain people have a predisposition to colon cancer; children are innately disposed to categorize objects in certain ways</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000040</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000016</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>material entity</t>
+          <t>disposition</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b140</t>
+          <t>(Elucidation) A disposition b is a realizable entity such that if b ceases to exist then its bearer is physically changed &amp; b's realization occurs when and because this bearer is in some special physical circumstances &amp; this realization occurs in virtue of the bearer's physical make-up</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000040</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000016</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>material entity</t>
+          <t>disposition</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b139</t>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000040</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000001</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>material entity</t>
+          <t>entity</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000141</t>
+          <t>Julius Caesar; the Second World War; your body mass index; Verdi's Requiem</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000030</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000001</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>entity</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000040</t>
+          <t>001-BFO</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000027</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000001</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>object aggregate</t>
+          <t>entity</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000040</t>
+          <t>(Elucidation) An entity is anything that exists or has existed or will exist</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000003</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000001</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>occurrent</t>
+          <t>entity</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000001</t>
+          <t>entity</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000026</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000001</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>one-dimensional spatial region</t>
+          <t>entity</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000006</t>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000026</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000142</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>one-dimensional spatial region</t>
+          <t>fiat line</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b110</t>
+          <t>fiat line</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000038</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000142</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>one-dimensional temporal region</t>
+          <t>fiat line</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b138</t>
+          <t>The Equator; all geopolitical boundaries; all lines of latitude and longitude; the median sulcus of your tongue; the line separating the outer surface of the mucosa of the lower lip from the outer surface of the skin of the chin</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000038</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000142</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>one-dimensional temporal region</t>
+          <t>fiat line</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000008</t>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000038</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000142</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>one-dimensional temporal region</t>
+          <t>fiat line</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000148</t>
+          <t>(Elucidation) A fiat line is a one-dimensional continuant fiat boundary that is continuous</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000038</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000142</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>one-dimensional temporal region</t>
+          <t>fiat line</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b134</t>
+          <t>032-BFO</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000015</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000142</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>process</t>
+          <t>fiat line</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b107</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000140</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000015</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000142</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>process</t>
+          <t>fiat line</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000003</t>
+          <t>n02f2337a1565431a8be6a3d794e45186b147</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000015</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000024</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>process</t>
+          <t>fiat object part</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b103</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000040</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000015</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000024</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>process</t>
+          <t>fiat object part</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b108</t>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000035</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000024</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>process boundary</t>
+          <t>fiat object part</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b126</t>
+          <t>027-BFO</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000035</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000024</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>process boundary</t>
+          <t>fiat object part</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b130</t>
+          <t>fiat object part</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000035</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000024</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>process boundary</t>
+          <t>fiat object part</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b124</t>
+          <t>The upper and lower lobes of the left lung; the dorsal and ventral surfaces of the body; the Western hemisphere of the Earth; the FMA:regional parts of an intact human body</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000035</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000024</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>process boundary</t>
+          <t>fiat object part</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b125</t>
+          <t>(Elucidation) A fiat object part b is a material entity &amp; such that if b exists then it is continuant part of some object c &amp; demarcated from the remainder of c by one or more fiat surfaces</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000035</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000147</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>process boundary</t>
+          <t>fiat point</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000003</t>
+          <t>031-BFO</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000019</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000147</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>quality</t>
+          <t>fiat point</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000020</t>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000017</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000147</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>realizable entity</t>
+          <t>fiat point</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000019</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000140</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000017</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000147</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>realizable entity</t>
+          <t>fiat point</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000020</t>
+          <t>The geographic North Pole; the quadripoint where the boundaries of Colorado, Utah, New Mexico and Arizona meet; the point of origin of some spatial coordinate system</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000145</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000147</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>relational quality</t>
+          <t>fiat point</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000019</t>
+          <t>n02f2337a1565431a8be6a3d794e45186b152</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000023</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000147</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>role</t>
+          <t>fiat point</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000017</t>
+          <t>fiat point</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000029</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000147</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>site</t>
+          <t>fiat point</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000141</t>
+          <t>(Elucidation) A fiat point is a zero-dimensional continuant fiat boundary that consists of a single point</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000029</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000146</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>site</t>
+          <t>fiat surface</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b123</t>
+          <t>(Elucidation) A fiat surface is a two-dimensional continuant fiat boundary that is self-connected</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000029</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000146</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>site</t>
+          <t>fiat surface</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b119</t>
+          <t>fiat surface</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000029</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000146</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>site</t>
+          <t>fiat surface</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b115</t>
+          <t>n02f2337a1565431a8be6a3d794e45186b151</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000006</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000146</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>spatial region</t>
+          <t>fiat surface</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000141</t>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000006</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000146</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>spatial region</t>
+          <t>fiat surface</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b93</t>
+          <t>033-BFO</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000011</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000146</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>spatiotemporal region</t>
+          <t>fiat surface</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b102</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000140</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000011</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000146</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>spatiotemporal region</t>
+          <t>fiat surface</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000003</t>
+          <t>The surface of the Earth; the plane separating the smoking from the non-smoking zone in a restaurant</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000011</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000034</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>spatiotemporal region</t>
+          <t>function</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b101</t>
+          <t>064-BFO</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000020</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000034</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>specifically dependent continuant</t>
+          <t>function</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000002</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000016</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000203</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000034</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>temporal instant</t>
+          <t>function</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000148</t>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000202</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000034</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>temporal interval</t>
+          <t>function</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000038</t>
+          <t>The function of a hammer to drive in nails; the function of a heart pacemaker to regulate the beating of a heart through electricity</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000008</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000034</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>temporal region</t>
+          <t>function</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b95</t>
+          <t>function</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000008</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000034</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>temporal region</t>
+          <t>function</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000003</t>
+          <t>(Elucidation) A function is a disposition that exists in virtue of its bearer's physical make-up &amp; this physical make-up is something the bearer possesses because it came into being either through evolution (in the case of natural biological entities) or through intentional design (in the case of artefacts) in order to realize processes of a certain sort</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000008</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000031</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>temporal region</t>
+          <t>generically dependent continuant</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b94</t>
+          <t>generically dependent continuant</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000028</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000031</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>three-dimensional spatial region</t>
+          <t>generically dependent continuant</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000006</t>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000028</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000031</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>three-dimensional spatial region</t>
+          <t>generically dependent continuant</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b114</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000002</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000009</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000031</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>two-dimensional spatial region</t>
+          <t>generically dependent continuant</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000006</t>
+          <t>(Elucidation) A generically dependent continuant is an entity that exists in virtue of the fact that there is at least one of what may be multiple copies which is the content or the pattern that multiple copies would share</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000009</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000031</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>two-dimensional spatial region</t>
+          <t>generically dependent continuant</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b96</t>
+          <t>074-BFO</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000018</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000031</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>zero-dimensional spatial region</t>
+          <t>generically dependent continuant</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b109</t>
+          <t>The pdf file on your laptop; the pdf file that is a copy thereof on my laptop; the sequence of this protein molecule; the sequence that is a copy thereof in that protein molecule; the content that is shared by a string of dots and dashes written on a page and the transmitted Morse code signal; the content of a sentence; an engineering blueprint</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000018</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000031</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>zero-dimensional spatial region</t>
+          <t>generically dependent continuant</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000006</t>
+          <t>g-dependent continuant</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/BFO_0000148</t>
+          <t>http://purl.obolibrary.org/obo/BFO_0000182</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>zero-dimensional temporal region</t>
+          <t>history</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>n654591509ee5490b96b76adca86ca805b153</t>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000182</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>history</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>The life of an organism from the beginning to the end of its existence</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000182</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>history</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>(Elucidation) A history is a process that is the sum of the totality of processes taking place in the spatiotemporal region occupied by the material part of a material entity</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000182</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>history</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>history</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000182</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>history</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>138-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000182</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>history</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000015</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000141</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>immaterial entity</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>b is an immaterial entity =Def b is an independent continuant which is such that there is no time t when it has a material entity as continuant part</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000141</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>immaterial entity</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>028-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000141</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>immaterial entity</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000141</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>immaterial entity</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>As for fiat point, fiat line, fiat surface, site</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000141</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>immaterial entity</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000004</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000141</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>immaterial entity</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>immaterial entity</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000004</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>independent continuant</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>017-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000004</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>independent continuant</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b92</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000004</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>independent continuant</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000002</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000004</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>independent continuant</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>independent continuant</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000004</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>independent continuant</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000004</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>independent continuant</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>b is an independent continuant =Def b is a continuant &amp; there is no c such that b specifically depends on c or b generically depends on c</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000004</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>independent continuant</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>An atom; a molecule; an organism; a heart; a chair; the bottom right portion of a human torso; a leg; the interior of your mouth; a spatial region; an orchestra</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000040</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>material entity</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>A human being; the undetached arm of a human being; an aggregate of human beings</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000040</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>material entity</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b140</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000040</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>material entity</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000004</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000040</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>material entity</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>material entity</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000040</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>material entity</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>019-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000040</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>material entity</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b139</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000040</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>material entity</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000040</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>material entity</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>(Elucidation) A material entity is an independent continuant that at all times at which it exists has some portion of matter as continuant part</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000040</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>material entity</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000141</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000030</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000040</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000030</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000030</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000030</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>A description of three primary sorts of causal unity is provided in Basic Formal Ontology 2.0. Specification and User Guide</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000030</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>An organism; a fish tank; a planet; a laptop; a valve; a block of marble; an ice cube</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000030</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>(Elucidation) An object is a material entity which manifests causal unity &amp; is of a type instances of which are maximal relative to the sort of causal unity manifested</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000030</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>024-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000027</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>object aggregate</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000040</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000027</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>object aggregate</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000027</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>object aggregate</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>object aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000027</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>object aggregate</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>025-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000027</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>object aggregate</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>The aggregate of the musicians in a symphony orchestra and their instruments; the aggregate of bearings in a constant velocity axle joint; the nitrogen atoms in the atmosphere; a collection of cells in a blood biobank</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000027</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>object aggregate</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>'Exactly' means that there are no parts of the object aggregate other than its member parts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000027</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>object aggregate</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>The unit can, at certain times, consist of exactly one object, for example, when a wolf litter loses all but one of its pups, but it must at some time have a plurality of member parts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000027</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>object aggregate</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>(Elucidation) An object aggregate is a material entity consisting exactly of a plurality (≥1) of objects as member parts which together form a unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000003</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>occurrent</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>occurrent</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000003</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>occurrent</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000003</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>occurrent</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>077-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000003</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>occurrent</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>As for process, history, process boundary, spatiotemporal region, zero-dimensional temporal region, one-dimensional temporal region, temporal interval, temporal instant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000003</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>occurrent</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000001</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000003</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>occurrent</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>(Elucidation) An occurrent is an entity that unfolds itself in time or it is the start or end of such an entity or it is a temporal or spatiotemporal region</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000026</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>one-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>An edge of a cube-shaped portion of space; a line connecting two points; two parallel lines extended in space</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000026</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>one-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000006</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000026</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>one-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>038-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000026</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>one-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>one-dimensional spatial region</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000026</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>one-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b110</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000026</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>one-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>(Elucidation) A one-dimensional spatial region is a whole consisting of a line together with zero or more lines which may have points as parts</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000026</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>one-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000038</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>one-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>The temporal region during which a process occurs</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000038</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>one-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>(Elucidation) A one-dimensional temporal region is a temporal region that is a whole that has a temporal interval and zero or more temporal intervals and temporal instants as parts</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000038</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>one-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b134</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000038</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>one-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000008</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000038</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>one-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b138</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000038</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>one-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>103-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000038</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>one-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>one-dimensional temporal region</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000038</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>one-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000038</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>one-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
           <t>http://purl.obolibrary.org/obo/BFO_0000148</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000015</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>(Elucidation) p is a process means p is an occurrent that has some temporal proper part and for some time t, p has some material entity as participant</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000015</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000015</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>083-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000015</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000003</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000015</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000015</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>An act of selling; the life of an organism; a process of sleeping; a process of cell-division; a beating of the heart; a process of meiosis; the taxiing of an aircraft; the programming of a computer</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000015</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b103</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000015</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b108</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000015</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000015</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b107</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000035</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>process boundary</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b126</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000035</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>process boundary</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>084-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000035</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>process boundary</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>process boundary</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000035</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>process boundary</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000035</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>process boundary</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>The boundary between the 2nd and 3rd year of your life</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000035</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>process boundary</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>p is a process boundary =Def p is a temporal part of a process &amp; p has no proper temporal parts</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000035</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>process boundary</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b125</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000035</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>process boundary</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b130</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000035</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>process boundary</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b124</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000035</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>process boundary</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000003</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000019</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>quality</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>quality</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000019</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>quality</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000019</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>quality</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>(Elucidation) A quality is a specifically dependent continuant that, in contrast to roles and dispositions, does not require any further process in order to be realized</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000019</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>quality</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>055-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000019</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>quality</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000020</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000019</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>quality</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>The colour of a tomato; the ambient temperature of this portion of air; the length of the circumference of your waist; the shape of your nose; the shape of your nostril; the mass of this piece of gold</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000017</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>realizable entity</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000017</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>realizable entity</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000019</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000017</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>realizable entity</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>058-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000017</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>realizable entity</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000020</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000017</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>realizable entity</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>The role of being a doctor; the role of this boundary to delineate where Utah and Colorado meet; the function of your reproductive organs; the disposition of your blood to coagulate; the disposition of this piece of metal to conduct electricity</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000017</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>realizable entity</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>realizable entity</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000017</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>realizable entity</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>(Elucidation) A realizable entity is a specifically dependent continuant that inheres in some independent continuant which is not a spatial region &amp; which is of a type some instances of which are realized in processes of a correlated type</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000145</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>relational quality</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000019</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000145</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>relational quality</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>relational quality</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000145</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>relational quality</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>A marriage bond; an instance of love; an obligation between one person and another</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000145</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>relational quality</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>057-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000145</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>relational quality</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>b is a relational quality =Def b is a quality &amp; there exists c and d such that c and d are not identical &amp; b specifically depends on c &amp; b specifically depends on d</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000145</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>relational quality</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000023</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>externally-grounded realizable entity</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000023</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000023</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000017</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000023</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>(Elucidation) A role b is a realizable entity such that b exists because there is some single bearer that is in some special physical, social, or institutional set of circumstances in which this bearer does not have to be &amp; b is not such that, if it ceases to exist, then the physical make-up of the bearer is thereby changed</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000023</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000023</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>The priest role; the student role; the role of subject in a clinical trial; the role of a stone in marking a property boundary; the role of a boundary to demarcate two neighbouring administrative territories; the role of a building in serving as a military target</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000023</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>061-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000029</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b115</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000029</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000029</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000141</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000029</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>034-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000029</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b119</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000029</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>(Elucidation) A site is a three-dimensional immaterial entity whose boundaries either (partially or wholly) coincide with the boundaries of one or more material entities or have locations determined in relation to some material entity</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000029</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b123</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000029</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000029</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>A hole in a portion of cheese; a rabbit hole; the Grand Canyon; the Piazza San Marco; the kangaroo-joey-containing hole of a kangaroo pouch; your left nostril (a fiat part - the opening - of your left nasal cavity); the lumen of your gut; the hold of a ship; the interior of the trunk of your car; hole in an engineered floor joist</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000006</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>spatial region</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000006</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>spatial region</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>spatial region</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000006</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>spatial region</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>035-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000006</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>spatial region</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>As for zero-dimensional spatial region, one-dimensional spatial region, two-dimensional spatial region, three-dimensional spatial region</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000006</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>spatial region</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000141</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000006</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>spatial region</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>(Elucidation) A spatial region is a continuant entity that is a continuant part of the spatial projection of a portion of spacetime at a given time</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000006</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>spatial region</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b93</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000011</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>spatiotemporal region</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>095-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000011</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>spatiotemporal region</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>The spatiotemporal region occupied by the development of a cancer tumour; the spatiotemporal region occupied by an orbiting satellite</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000011</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>spatiotemporal region</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b102</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000011</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>spatiotemporal region</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>(Elucidation) A spatiotemporal region is an occurrent that is an occurrent part of spacetime</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000011</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>spatiotemporal region</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000003</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000011</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>spatiotemporal region</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>spatiotemporal region</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000011</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>spatiotemporal region</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>'Spacetime' here refers to the maximal instance of the universal spatiotemporal region.</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000011</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>spatiotemporal region</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000011</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>spatiotemporal region</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b101</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000020</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>specifically dependent continuant</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>b is a specifically dependent continuant =Def b is a continuant &amp; there is some independent continuant c which is not a spatial region &amp; which is such that b specifically depends on c</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000020</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>specifically dependent continuant</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>(with multiple bearers) John's love for Mary; the ownership relation between John and this statue; the relation of authority between John and his subordinates</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000020</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>specifically dependent continuant</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>specifically dependent continuant</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000020</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>specifically dependent continuant</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000002</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000020</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>specifically dependent continuant</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>050-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000020</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>specifically dependent continuant</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000020</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>specifically dependent continuant</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>(with one bearer) The mass of this tomato; the pink colour of a medium rare piece of grilled filet mignon at its centre; the smell of this portion of mozzarella; the disposition of this fish to decay; the role of being a doctor; the function of this heart to pump blood; the shape of this hole</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000203</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>temporal instant</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>(Elucidation) A temporal instant is a zero-dimensional temporal region that has no proper temporal part</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000203</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>temporal instant</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>The millennium</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000203</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>temporal instant</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000203</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>temporal instant</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>temporal instant</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000203</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>temporal instant</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000148</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000203</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>temporal instant</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>209-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000202</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>The year 2018.</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000202</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000038</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000202</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>155-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000202</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000202</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000202</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>(Elucidation) A temporal interval is a one-dimensional temporal region that is continuous, thus without gaps or breaks</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000202</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>temporal interval</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>A one-dimensional temporal region can include as parts not only temporal intervals but also temporal instants separated from other parts by gaps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000008</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>temporal region</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>temporal region</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000008</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>temporal region</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000008</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>temporal region</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>As for zero-dimensional temporal region and one-dimensional temporal region</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000008</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>temporal region</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b94</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000008</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>temporal region</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000003</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000008</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>temporal region</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b95</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000008</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>temporal region</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>(Elucidation) A temporal region is an occurrent over which processes can unfold</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000008</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>temporal region</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>100-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000028</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>three-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>three-dimensional spatial region</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000028</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>three-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000006</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000028</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>three-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>040-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000028</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>three-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>(Elucidation) A three-dimensional spatial region is a whole consisting of a spatial volume together with zero or more spatial volumes which may have spatial regions of lower dimension as parts</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000028</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>three-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b114</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000028</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>three-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>A cube-shaped region of space; a sphere-shaped region of space; the region of space occupied by all and only the planets in the solar system at some point in time</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000028</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>three-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000009</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>two-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000006</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000009</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>two-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>The surface of a sphere-shaped part of space; an infinitely thin plane in space</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000009</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>two-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b96</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000009</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>two-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>039-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000009</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>two-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>(Elucidation) A two-dimensional spatial region is a spatial region that is a whole consisting of a surface together with zero or more surfaces which may have spatial regions of lower dimension as parts</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000009</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>two-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>two-dimensional spatial region</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000009</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>two-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000018</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>zero-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000018</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>zero-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>037-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000018</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>zero-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>The spatial region occupied at some time instant by the North Pole</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000018</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>zero-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>zero-dimensional spatial region</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000018</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>zero-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b109</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000018</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>zero-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>(Elucidation) A zero-dimensional spatial region is one or a collection of more than one spatially disjoint points in space</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000018</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>zero-dimensional spatial region</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000006</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000148</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
         <is>
           <t>zero-dimensional temporal region</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>n02f2337a1565431a8be6a3d794e45186b153</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000148</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>zero-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>zero-dimensional temporal region</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000148</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>zero-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>http://www.w3.org/2002/07/owl#Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000148</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>zero-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>(Elucidation) A zero-dimensional temporal region is a temporal region that is a whole consisting of one or more separated temporal instants as parts</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000148</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>zero-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
         <is>
           <t>http://purl.obolibrary.org/obo/BFO_0000008</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000148</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>zero-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>102-BFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000148</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>zero-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>A temporal region that is occupied by a process boundary; the moment at which a finger is detached in an industrial accident</t>
         </is>
       </c>
     </row>

</xml_diff>